<commit_message>
working on utility and other reviewer comments
</commit_message>
<xml_diff>
--- a/data/byhand_typology-weights2.xlsx
+++ b/data/byhand_typology-weights2.xlsx
@@ -3,12 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35A47131-5B5C-47F3-B188-D1CB4D43DCF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FF5402A-1B16-46DF-8989-D49D759DD7AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="324" yWindow="1656" windowWidth="9684" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="12">
   <si>
     <t>Conservationist</t>
   </si>
@@ -73,7 +74,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -84,6 +85,12 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Aptos"/>
       <family val="2"/>
     </font>
@@ -108,13 +115,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -452,6 +462,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1881D26D-58E6-4B13-B3DA-2DFBBC0E86E2}">
   <dimension ref="A6:H11"/>
   <sheetFormatPr defaultColWidth="20.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
@@ -463,14 +483,14 @@
       <c r="C6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F6" t="s">
         <v>6</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>5</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>7</v>
@@ -483,22 +503,22 @@
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="1">
-        <v>40</v>
-      </c>
-      <c r="C7" s="1">
-        <v>20</v>
-      </c>
-      <c r="D7" s="1">
-        <v>15</v>
-      </c>
-      <c r="E7" s="1">
-        <v>10</v>
-      </c>
-      <c r="F7" s="1">
-        <v>5</v>
-      </c>
-      <c r="G7" s="1">
+      <c r="B7" s="3">
+        <v>50</v>
+      </c>
+      <c r="C7" s="3">
+        <v>10</v>
+      </c>
+      <c r="D7" s="3">
+        <v>10</v>
+      </c>
+      <c r="E7" s="3">
+        <v>10</v>
+      </c>
+      <c r="F7" s="3">
+        <v>10</v>
+      </c>
+      <c r="G7" s="3">
         <v>10</v>
       </c>
       <c r="H7">
@@ -510,23 +530,23 @@
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="1">
-        <v>40</v>
-      </c>
-      <c r="C8" s="1">
-        <v>40</v>
-      </c>
-      <c r="D8" s="1">
-        <v>7.5</v>
-      </c>
-      <c r="E8" s="1">
-        <v>7.5</v>
-      </c>
-      <c r="F8" s="1">
-        <v>0</v>
-      </c>
-      <c r="G8" s="1">
-        <v>5</v>
+      <c r="B8" s="3">
+        <v>70</v>
+      </c>
+      <c r="C8" s="3">
+        <v>15</v>
+      </c>
+      <c r="D8" s="3">
+        <v>15</v>
+      </c>
+      <c r="E8" s="3">
+        <v>0</v>
+      </c>
+      <c r="F8" s="3">
+        <v>0</v>
+      </c>
+      <c r="G8" s="3">
+        <v>0</v>
       </c>
       <c r="H8">
         <f t="shared" ref="H8:H10" si="0">SUM(B8:G8)</f>
@@ -537,23 +557,23 @@
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B9" s="1">
-        <v>50</v>
-      </c>
-      <c r="C9" s="1">
-        <v>40</v>
-      </c>
-      <c r="D9" s="1">
-        <v>0</v>
-      </c>
-      <c r="E9" s="1">
-        <v>5</v>
-      </c>
-      <c r="F9" s="1">
-        <v>0</v>
-      </c>
-      <c r="G9" s="1">
-        <v>5</v>
+      <c r="B9" s="3">
+        <v>20</v>
+      </c>
+      <c r="C9" s="3">
+        <v>30</v>
+      </c>
+      <c r="D9" s="3">
+        <v>10</v>
+      </c>
+      <c r="E9" s="3">
+        <v>10</v>
+      </c>
+      <c r="F9" s="3">
+        <v>20</v>
+      </c>
+      <c r="G9" s="3">
+        <v>10</v>
       </c>
       <c r="H9">
         <f t="shared" si="0"/>
@@ -564,22 +584,22 @@
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="1">
-        <v>60</v>
-      </c>
-      <c r="C10" s="1">
-        <v>40</v>
-      </c>
-      <c r="D10" s="1">
-        <v>0</v>
-      </c>
-      <c r="E10" s="1">
-        <v>0</v>
-      </c>
-      <c r="F10" s="1">
-        <v>0</v>
-      </c>
-      <c r="G10" s="1">
+      <c r="B10" s="3">
+        <v>90</v>
+      </c>
+      <c r="C10" s="3">
+        <v>0</v>
+      </c>
+      <c r="D10" s="3">
+        <v>10</v>
+      </c>
+      <c r="E10" s="3">
+        <v>0</v>
+      </c>
+      <c r="F10" s="3">
+        <v>0</v>
+      </c>
+      <c r="G10" s="3">
         <v>0</v>
       </c>
       <c r="H10">
@@ -596,22 +616,172 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E51CCD38-78BD-4099-8324-FD61C7834A5E}">
+  <dimension ref="B3:F10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="3" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="3">
+        <v>50</v>
+      </c>
+      <c r="D4" s="3">
+        <v>50</v>
+      </c>
+      <c r="E4" s="3">
+        <v>60</v>
+      </c>
+      <c r="F4" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="3">
+        <v>20</v>
+      </c>
+      <c r="D5" s="3">
+        <v>30</v>
+      </c>
+      <c r="E5" s="3">
+        <v>40</v>
+      </c>
+      <c r="F5" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="D6" s="3">
+        <v>10</v>
+      </c>
+      <c r="E6" s="3">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="D7" s="3">
+        <v>10</v>
+      </c>
+      <c r="E7" s="3">
+        <v>0</v>
+      </c>
+      <c r="F7" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="D8" s="3">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3">
+        <v>0</v>
+      </c>
+      <c r="F8" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="D9" s="3">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3">
+        <v>0</v>
+      </c>
+      <c r="F9" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B10" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10">
+        <f>SUM(C4:C9)</f>
+        <v>100</v>
+      </c>
+      <c r="D10">
+        <f>SUM(D4:D9)</f>
+        <v>100</v>
+      </c>
+      <c r="E10">
+        <f>SUM(E4:E9)</f>
+        <v>100</v>
+      </c>
+      <c r="F10">
+        <f>SUM(F4:F9)</f>
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"blankspreadsheet","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"blankspreadsheet","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7408D0D6-C97A-426B-8466-DDDAA7A3F420}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{613AEFFE-C095-42A7-A0AC-5564FFC1D197}">
   <ds:schemaRefs/>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7408D0D6-C97A-426B-8466-DDDAA7A3F420}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
 </file>
</xml_diff>